<commit_message>
chore: reorganizacion de funcion abolladura en 004_runExperimentos
</commit_message>
<xml_diff>
--- a/Resultados/todos_los_resultados.xlsx
+++ b/Resultados/todos_los_resultados.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="4342" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="4352" uniqueCount="19">
   <si>
     <t>ID</t>
   </si>
@@ -531,22 +531,22 @@
         <v>5</v>
       </c>
       <c r="D2" s="0">
-        <v>1526.1153978</v>
+        <v>124.556647</v>
       </c>
       <c r="E2" s="0">
-        <v>0.31274670186575654</v>
+        <v>0.16273530884157902</v>
       </c>
       <c r="F2" s="0" t="b">
         <v>1</v>
       </c>
       <c r="G2" s="0">
-        <v>10.263452121309435</v>
+        <v>7.3096821824949494</v>
       </c>
       <c r="H2" s="0">
-        <v>9.6639832282444669</v>
+        <v>7.0272769983188006</v>
       </c>
       <c r="I2" s="0">
-        <v>10.263452121309435</v>
+        <v>7.3096821824949494</v>
       </c>
       <c r="J2" s="0">
         <v>1</v>

</xml_diff>

<commit_message>
feat: integrado correcamente la corrosion
</commit_message>
<xml_diff>
--- a/Resultados/todos_los_resultados.xlsx
+++ b/Resultados/todos_los_resultados.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="4352" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="4422" uniqueCount="19">
   <si>
     <t>ID</t>
   </si>
@@ -525,31 +525,31 @@
         <v>1</v>
       </c>
       <c r="B2" s="0">
-        <v>1</v>
+        <v>71</v>
       </c>
       <c r="C2" s="0">
-        <v>5</v>
+        <v>49</v>
       </c>
       <c r="D2" s="0">
-        <v>124.556647</v>
+        <v>5264.6146160999997</v>
       </c>
       <c r="E2" s="0">
-        <v>0.16273530884157902</v>
+        <v>1.9498492516911063</v>
       </c>
       <c r="F2" s="0" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G2" s="0">
-        <v>7.3096821824949494</v>
+        <v>29.475855614814282</v>
       </c>
       <c r="H2" s="0">
-        <v>7.0272769983188006</v>
+        <v>13.323921996693983</v>
       </c>
       <c r="I2" s="0">
-        <v>7.3096821824949494</v>
+        <v>29.475855614814282</v>
       </c>
       <c r="J2" s="0">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="K2" t="s">
         <v>11</v>

</xml_diff>